<commit_message>
fix(build): make the workbook build independent of optional lxml
openpyxl serializes XML differently when lxml is installed, so CI (no lxml)
rebuilt different bytes and W11 failed. The builder now forces openpyxl's
standard writer and refuses to build if lxml serialization is active.
Regression test: test_build_does_not_depend_on_optional_lxml.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LZw4KSKXtfqrAUNK4GcNxe
</commit_message>
<xml_diff>
--- a/workbook/implementation-tracker-workbook.xlsx
+++ b/workbook/implementation-tracker-workbook.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phases and Gates" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requests and Handoffs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escalation Rules" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks and Issues" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness Scorecard" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity Inputs" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Log" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Summary" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Lookups" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Projects" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Phases and Gates" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Tasks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Requests and Handoffs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Escalation Rules" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Risks and Issues" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Readiness Scorecard" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Capacity Inputs" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Event Log" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="KPI Summary" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="calculation_as_of_at">'README'!$D$10</definedName>
@@ -290,13 +290,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -320,7 +320,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -360,8 +360,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -399,9 +399,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
docs(publication): prepare R3 0.1.0 for joint publication review
Widen columns so no header splits mid-word and free text is readable, and
make the KPI chart count whole projects. Add two README screenshots
rendered from the bundled synthetic workbook by tools/render_screenshots.py,
the R1/R3 relationship on the first screen, a navigation map, an author
line, and a plain Excel limitation. Store the R30 vendor list as SHA-256
hashes, with matcher tests. Record the strict gate result.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LZw4KSKXtfqrAUNK4GcNxe
</commit_message>
<xml_diff>
--- a/workbook/implementation-tracker-workbook.xlsx
+++ b/workbook/implementation-tracker-workbook.xlsx
@@ -354,6 +354,7 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <min val="0"/>
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
@@ -372,9 +373,11 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <majorUnit val="1"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -1309,7 +1312,7 @@
     <col width="2" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1767,25 +1770,25 @@
   <dimension ref="A1:W39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="31" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="29" customWidth="1" min="19" max="19"/>
     <col width="36" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="60" customWidth="1" min="23" max="23"/>
@@ -5161,18 +5164,18 @@
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="27" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8211,16 +8214,16 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
     <col width="60" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
@@ -9193,22 +9196,22 @@
   <dimension ref="A1:W173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
     <col width="60" customWidth="1" min="12" max="12"/>
     <col width="32" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
     <col width="26" customWidth="1" min="19" max="19"/>
     <col width="30" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
@@ -16407,24 +16410,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
     <col width="22" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
@@ -16881,43 +16884,43 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
     <col width="24" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="21" customWidth="1" min="27" max="27"/>
     <col width="14" customWidth="1" min="28" max="28"/>
     <col width="14" customWidth="1" min="29" max="29"/>
     <col width="14" customWidth="1" min="30" max="30"/>
     <col width="14" customWidth="1" min="31" max="31"/>
     <col width="20" customWidth="1" min="32" max="32"/>
-    <col width="14" customWidth="1" min="33" max="33"/>
-    <col width="14" customWidth="1" min="34" max="34"/>
-    <col width="14" customWidth="1" min="35" max="35"/>
-    <col width="14" customWidth="1" min="36" max="36"/>
+    <col width="21" customWidth="1" min="33" max="33"/>
+    <col width="26" customWidth="1" min="34" max="34"/>
+    <col width="16" customWidth="1" min="35" max="35"/>
+    <col width="17" customWidth="1" min="36" max="36"/>
     <col width="40" customWidth="1" min="37" max="37"/>
-    <col width="14" customWidth="1" min="38" max="38"/>
-    <col width="14" customWidth="1" min="39" max="39"/>
-    <col width="14" customWidth="1" min="40" max="40"/>
-    <col width="14" customWidth="1" min="41" max="41"/>
+    <col width="17" customWidth="1" min="38" max="38"/>
+    <col width="16" customWidth="1" min="39" max="39"/>
+    <col width="17" customWidth="1" min="40" max="40"/>
+    <col width="18" customWidth="1" min="41" max="41"/>
     <col width="20" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
@@ -18847,21 +18850,21 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
     <col width="26" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
@@ -21567,39 +21570,39 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="23" customWidth="1" min="17" max="17"/>
+    <col width="23" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
     <col width="28" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="15" customWidth="1" min="26" max="26"/>
     <col width="14" customWidth="1" min="27" max="27"/>
-    <col width="18" customWidth="1" min="28" max="28"/>
-    <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="25" customWidth="1" min="28" max="28"/>
+    <col width="17" customWidth="1" min="29" max="29"/>
     <col width="20" customWidth="1" min="30" max="30"/>
     <col width="20" customWidth="1" min="31" max="31"/>
-    <col width="14" customWidth="1" min="32" max="32"/>
-    <col width="14" customWidth="1" min="33" max="33"/>
-    <col width="14" customWidth="1" min="34" max="34"/>
-    <col width="18" customWidth="1" min="35" max="35"/>
-    <col width="16" customWidth="1" min="36" max="36"/>
+    <col width="23" customWidth="1" min="32" max="32"/>
+    <col width="17" customWidth="1" min="33" max="33"/>
+    <col width="15" customWidth="1" min="34" max="34"/>
+    <col width="19" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
     <col width="22" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
@@ -22727,18 +22730,18 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
     <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
     <col width="70" customWidth="1" min="15" max="15"/>
     <col width="34" customWidth="1" min="16" max="16"/>
   </cols>
@@ -23744,34 +23747,34 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="34" customWidth="1" min="23" max="23"/>
-    <col width="40" customWidth="1" min="24" max="24"/>
+    <col width="44" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
     <col width="20" customWidth="1" min="28" max="28"/>
     <col width="20" customWidth="1" min="29" max="29"/>
     <col width="34" customWidth="1" min="30" max="30"/>
-    <col width="14" customWidth="1" min="31" max="31"/>
-    <col width="14" customWidth="1" min="32" max="32"/>
-    <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="17" customWidth="1" min="31" max="31"/>
+    <col width="17" customWidth="1" min="32" max="32"/>
+    <col width="18" customWidth="1" min="33" max="33"/>
     <col width="22" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
@@ -24858,31 +24861,31 @@
   <dimension ref="A1:AB22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
-    <col width="10" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="34" customWidth="1" min="26" max="26"/>
     <col width="60" customWidth="1" min="27" max="27"/>
     <col width="22" customWidth="1" min="28" max="28"/>
   </cols>

</xml_diff>